<commit_message>
made some changes to parameter data and horizontal K spreadsheets
</commit_message>
<xml_diff>
--- a/gsflow/horizontal_K_from_Amod.xlsx
+++ b/gsflow/horizontal_K_from_Amod.xlsx
@@ -14,7 +14,7 @@
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="140000" concurrentCalc="0"/>
+  <calcPr calcId="152511"/>
   <extLst>
     <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{7523E5D3-25F3-A5E0-1632-64F254C22452}">
       <mx:ArchID Flags="2"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="13">
   <si>
     <t>m/s</t>
   </si>
@@ -60,6 +60,9 @@
   </si>
   <si>
     <t>Units</t>
+  </si>
+  <si>
+    <t>ft/s</t>
   </si>
 </sst>
 </file>
@@ -92,24 +95,31 @@
     </font>
     <font>
       <sz val="14"/>
-      <color rgb="FF222222"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="14"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="14"/>
+      <color rgb="FF222222"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -134,12 +144,20 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="11" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="1" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="11" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="11" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="11">
     <cellStyle name="Followed Hyperlink" xfId="2" builtinId="9" hidden="1"/>
@@ -489,136 +507,253 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="18.375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="18.375" customWidth="1"/>
+    <col min="5" max="5" width="13.625" customWidth="1"/>
+    <col min="6" max="6" width="11.625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:6" s="6" customFormat="1" ht="39" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="5" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A2" s="2">
+      <c r="A2" s="1">
         <v>1</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="D2" s="3">
+      <c r="D2" s="7">
         <v>0.01</v>
       </c>
-      <c r="E2" s="3">
+      <c r="E2" s="7">
         <v>5.9999999999999995E-4</v>
       </c>
-      <c r="F2" s="1">
+      <c r="F2" s="8">
         <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A3" s="2">
+      <c r="A3" s="1">
+        <v>1</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" s="7">
+        <f>D2*3.28084</f>
+        <v>3.2808400000000001E-2</v>
+      </c>
+      <c r="E3" s="7">
+        <f>E2*3.28084</f>
+        <v>1.9685039999999998E-3</v>
+      </c>
+      <c r="F3" s="7">
+        <f>F2*3.28084</f>
+        <v>6.56168</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A4" s="1">
         <v>2</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B4" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C4" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="D3" s="3">
+      <c r="D4" s="7">
         <v>4.0000000000000002E-4</v>
       </c>
-      <c r="E3" s="3">
+      <c r="E4" s="3">
         <v>4.0000000000000003E-5</v>
       </c>
-      <c r="F3" s="3">
+      <c r="F4" s="7">
         <v>1E-3</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="18" x14ac:dyDescent="0.25">
-      <c r="A4" s="4">
+    <row r="5" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A5" s="1">
+        <v>2</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D5" s="7">
+        <f>D4*3.28084</f>
+        <v>1.3123360000000001E-3</v>
+      </c>
+      <c r="E5" s="3">
+        <f>E4*3.28084</f>
+        <v>1.3123360000000001E-4</v>
+      </c>
+      <c r="F5" s="7">
+        <f>F4*3.28084</f>
+        <v>3.2808400000000001E-3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A6" s="4">
         <v>3</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B6" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C6" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="D4" s="3">
+      <c r="D6" s="7">
         <v>3.0000000000000001E-3</v>
       </c>
-      <c r="E4" s="3">
+      <c r="E6" s="3">
         <v>1E-4</v>
       </c>
-      <c r="F4" s="3">
+      <c r="F6" s="7">
         <v>0.02</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="18" x14ac:dyDescent="0.25">
-      <c r="A5" s="4">
+    <row r="7" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A7" s="4">
+        <v>3</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D7" s="7">
+        <f>D6*3.28084</f>
+        <v>9.8425200000000004E-3</v>
+      </c>
+      <c r="E7" s="3">
+        <f>E6*3.28084</f>
+        <v>3.2808400000000003E-4</v>
+      </c>
+      <c r="F7" s="7">
+        <f>F6*3.28084</f>
+        <v>6.5616800000000003E-2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A8" s="4">
         <v>4</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B8" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C8" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="D5" s="3">
+      <c r="D8" s="3">
         <v>4.9999999999999998E-8</v>
       </c>
-      <c r="E5" s="3">
+      <c r="E8" s="3">
         <v>5.0000000000000001E-9</v>
       </c>
-      <c r="F5" s="3">
+      <c r="F8" s="3">
         <v>4.9999999999999998E-7</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="18" x14ac:dyDescent="0.25">
-      <c r="A6" s="4">
+    <row r="9" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A9" s="4">
+        <v>4</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D9" s="3">
+        <f>D8*3.28084</f>
+        <v>1.6404199999999998E-7</v>
+      </c>
+      <c r="E9" s="3">
+        <f>E8*3.28084</f>
+        <v>1.64042E-8</v>
+      </c>
+      <c r="F9" s="3">
+        <f>F8*3.28084</f>
+        <v>1.6404199999999999E-6</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A10" s="4">
         <v>5</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B10" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C10" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="D6" s="3">
+      <c r="D10" s="3">
         <v>4.9999999999999999E-13</v>
       </c>
-      <c r="E6" s="1">
+      <c r="E10" s="2">
         <v>0</v>
       </c>
-      <c r="F6" s="3">
+      <c r="F10" s="3">
         <v>5.0000000000000002E-11</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A11" s="4">
+        <v>5</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D11" s="3">
+        <f t="shared" ref="D11:F11" si="0">D10*3.28084</f>
+        <v>1.64042E-12</v>
+      </c>
+      <c r="E11" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F11" s="3">
+        <f t="shared" si="0"/>
+        <v>1.64042E-10</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967292" verticalDpi="4294967292"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967292" verticalDpi="4294967292" r:id="rId1"/>
   <extLst>
     <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{64002731-A6B0-56B0-2670-7721B7C09600}">
       <mx:PLV Mode="0" OnePage="0" WScale="0"/>

</xml_diff>